<commit_message>
test(qa): ejecutar casos de revisión y actualizar documentación
Ejecuta MVC-GEN-05 en Chromium, Firefox y WebKit y registra las
revisiones de MVC-GEN-03 (bloqueado sin acceso a Figma), MVC-GEN-04,
SW-09 y ENT-12. Agrega DEF-09 a DEF-11 y actualiza la matriz, la
sección 3.9 y los README de QA. Los generadores ignoran las copias de
sincronización con sufijo " 2".
</commit_message>
<xml_diff>
--- a/QA/Matriz_Pruebas_Laboratorio1_QA.xlsx
+++ b/QA/Matriz_Pruebas_Laboratorio1_QA.xlsx
@@ -2725,7 +2725,7 @@
       </c>
       <c r="B7" s="6">
         <f>COUNTIF('Casos de prueba'!$K$2:$K$500,"Aprobado")</f>
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -2734,7 +2734,7 @@
       </c>
       <c r="B8" s="6">
         <f>COUNTIF('Casos de prueba'!$K$2:$K$500,"Fallido")</f>
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B9" s="6">
         <f>COUNTIF('Casos de prueba'!$K$2:$K$500,"Bloqueado")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -2752,7 +2752,7 @@
       </c>
       <c r="B10" s="6">
         <f>COUNTIF('Casos de prueba'!$K$2:$K$500,"Pendiente")</f>
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -2770,7 +2770,7 @@
       </c>
       <c r="B12" s="7">
         <f>IFERROR((B7+B8)/(B6-B11),0)</f>
-        <v>0.957575757575758</v>
+        <v>0.981818181818182</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -2779,7 +2779,7 @@
       </c>
       <c r="B13" s="7">
         <f>IFERROR(B7/(B7+B8),0)</f>
-        <v>0.930379746835443</v>
+        <v>0.919753086419753</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="B14" s="6">
         <f>COUNTIF(Defectos!$A$2:$A$500,"DEF-*")</f>
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -2797,7 +2797,7 @@
       </c>
       <c r="B15" s="6">
         <f>COUNTIFS(Defectos!$A$2:$A$500,"DEF-*",Defectos!$J$2:$J$500,"Abierto")+COUNTIFS(Defectos!$A$2:$A$500,"DEF-*",Defectos!$J$2:$J$500,"En corrección")</f>
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -2929,11 +2929,11 @@
       </c>
       <c r="D23" s="9">
         <f>COUNTIFS('Casos de prueba'!$C$2:$C$500,A23,'Casos de prueba'!$K$2:$K$500,"Fallido")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E23" s="9">
         <f>COUNTIFS('Casos de prueba'!$C$2:$C$500,A23,'Casos de prueba'!$K$2:$K$500,"Pendiente")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F23" s="9">
         <f>COUNTIFS('Casos de prueba'!$C$2:$C$500,A23,'Casos de prueba'!$K$2:$K$500,"Bloqueado")</f>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="C24" s="9">
         <f>COUNTIFS('Casos de prueba'!$C$2:$C$500,A24,'Casos de prueba'!$K$2:$K$500,"Aprobado")</f>
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D24" s="9">
         <f>COUNTIFS('Casos de prueba'!$C$2:$C$500,A24,'Casos de prueba'!$K$2:$K$500,"Fallido")</f>
@@ -2962,15 +2962,15 @@
       </c>
       <c r="E24" s="9">
         <f>COUNTIFS('Casos de prueba'!$C$2:$C$500,A24,'Casos de prueba'!$K$2:$K$500,"Pendiente")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F24" s="9">
         <f>COUNTIFS('Casos de prueba'!$C$2:$C$500,A24,'Casos de prueba'!$K$2:$K$500,"Bloqueado")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24" s="10">
         <f t="shared" si="0"/>
-        <v>0.775</v>
+        <v>0.825</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -3016,11 +3016,11 @@
       </c>
       <c r="D26" s="9">
         <f>COUNTIFS('Casos de prueba'!$C$2:$C$500,A26,'Casos de prueba'!$K$2:$K$500,"Fallido")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E26" s="9">
         <f>COUNTIFS('Casos de prueba'!$C$2:$C$500,A26,'Casos de prueba'!$K$2:$K$500,"Pendiente")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F26" s="9">
         <f>COUNTIFS('Casos de prueba'!$C$2:$C$500,A26,'Casos de prueba'!$K$2:$K$500,"Bloqueado")</f>
@@ -3041,23 +3041,23 @@
       </c>
       <c r="C27" s="12">
         <f>SUM(C20:C26)</f>
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D27" s="12">
         <f>SUM(D20:D26)</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E27" s="12">
         <f>SUM(E20:E26)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F27" s="12">
         <f>SUM(F20:F26)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G27" s="13">
         <f t="shared" si="0"/>
-        <v>0.890909090909091</v>
+        <v>0.903030303030303</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -3395,15 +3395,15 @@
       </c>
       <c r="G7" s="15">
         <f>COUNTIFS('Casos de prueba'!$B$2:$B$500,A7,'Casos de prueba'!$K$2:$K$500,"Fallido")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H7" s="15">
         <f>COUNTIFS('Casos de prueba'!$B$2:$B$500,A7,'Casos de prueba'!$K$2:$K$500,"Pendiente")+COUNTIFS('Casos de prueba'!$B$2:$B$500,A7,'Casos de prueba'!$K$2:$K$500,"Bloqueado")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I7" s="15" t="str">
         <f t="shared" si="0"/>
-        <v>En curso</v>
+        <v>Con fallos</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="27.95">
@@ -3425,7 +3425,7 @@
       </c>
       <c r="F8" s="15">
         <f>COUNTIFS('Casos de prueba'!$B$2:$B$500,A8,'Casos de prueba'!$K$2:$K$500,"Aprobado")</f>
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G8" s="15">
         <f>COUNTIFS('Casos de prueba'!$B$2:$B$500,A8,'Casos de prueba'!$K$2:$K$500,"Fallido")</f>
@@ -3433,7 +3433,7 @@
       </c>
       <c r="H8" s="15">
         <f>COUNTIFS('Casos de prueba'!$B$2:$B$500,A8,'Casos de prueba'!$K$2:$K$500,"Pendiente")+COUNTIFS('Casos de prueba'!$B$2:$B$500,A8,'Casos de prueba'!$K$2:$K$500,"Bloqueado")</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I8" s="15" t="str">
         <f t="shared" si="0"/>
@@ -3565,11 +3565,11 @@
       </c>
       <c r="G12" s="15">
         <f>COUNTIFS('Casos de prueba'!$B$2:$B$500,A12,'Casos de prueba'!$K$2:$K$500,"Fallido")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H12" s="15">
         <f>COUNTIFS('Casos de prueba'!$B$2:$B$500,A12,'Casos de prueba'!$K$2:$K$500,"Pendiente")+COUNTIFS('Casos de prueba'!$B$2:$B$500,A12,'Casos de prueba'!$K$2:$K$500,"Bloqueado")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I12" s="15" t="str">
         <f t="shared" si="0"/>
@@ -9901,16 +9901,30 @@
       </c>
       <c r="K106" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pendiente</t>
-        </is>
-      </c>
-      <c r="L106" s="17"/>
-      <c r="M106" s="17"/>
-      <c r="N106" s="18"/>
-      <c r="O106" s="17"/>
+          <t xml:space="preserve">Fallido</t>
+        </is>
+      </c>
+      <c r="L106" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Las 20 operaciones se agrupan por recurso y documentan sus códigos, pero ninguna tiene resumen ni descripción, y ninguna de las 15 propiedades de los DTO se describe. Campos como cc, ccPer, des, duenio, idProf, nom no se explican.</t>
+        </is>
+      </c>
+      <c r="M106" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EV-SW-01.png, EV-SW-09.txt</t>
+        </is>
+      </c>
+      <c r="N106" s="18">
+        <v>46322</v>
+      </c>
+      <c r="O106" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Automatizado</t>
+        </is>
+      </c>
       <c r="P106" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Revisión manual pendiente. Dato para la revisión: las operaciones no tienen summary ni descripciones porque el proyecto no genera el archivo XML de documentación.</t>
+          <t xml:space="preserve">El código ya tiene 4 comentarios /// &lt;summary&gt; en los DTO, pero el proyecto no genera el archivo XML de documentación, por lo que Swagger no los muestra. Revisión asistida: confirmar el criterio con el responsable de QA. Defecto DEF-10.</t>
         </is>
       </c>
     </row>
@@ -11891,16 +11905,30 @@
       </c>
       <c r="K141" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pendiente</t>
-        </is>
-      </c>
-      <c r="L141" s="17"/>
-      <c r="M141" s="17"/>
-      <c r="N141" s="18"/>
-      <c r="O141" s="17"/>
+          <t xml:space="preserve">Bloqueado</t>
+        </is>
+      </c>
+      <c r="L141" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No se pudo abrir el diseño de Figma desde el entorno de pruebas (requiere sesión o permiso del autor).</t>
+        </is>
+      </c>
+      <c r="M141" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pantallas/EV-MVC-GEN-03-*.png, EV-MVC-GEN-03.txt</t>
+        </is>
+      </c>
+      <c r="N141" s="18">
+        <v>46322</v>
+      </c>
+      <c r="O141" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Automatizado</t>
+        </is>
+      </c>
       <c r="P141" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Revisión manual pendiente: comparar con Figma las 21 capturas de evidencias/pantallas/EV-MVC-GEN-03-*.png.</t>
+          <t xml:space="preserve">Las 21 capturas de las pantallas implementadas están listas. Falta el enlace compartido de Figma o las exportaciones de Andrés para completar la comparación.</t>
         </is>
       </c>
     </row>
@@ -11937,16 +11965,30 @@
       </c>
       <c r="K142" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pendiente</t>
-        </is>
-      </c>
-      <c r="L142" s="17"/>
-      <c r="M142" s="17"/>
-      <c r="N142" s="18"/>
-      <c r="O142" s="17"/>
+          <t xml:space="preserve">Aprobado</t>
+        </is>
+      </c>
+      <c r="L142" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En 1366, 768 y 375 px ninguna página desborda horizontalmente; en tableta y móvil el menú lateral pasa a la parte superior, los formularios quedan en una columna y las tablas se desplazan dentro de su contenedor. El texto es legible (letra mínima 12 px).</t>
+        </is>
+      </c>
+      <c r="M142" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EV-MVC-GEN-04-*.png, EV-MVC-GEN-04-resumen-vacio.png, EV-MVC-GEN-04.txt</t>
+        </is>
+      </c>
+      <c r="N142" s="18">
+        <v>46322</v>
+      </c>
+      <c r="O142" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Automatizado</t>
+        </is>
+      </c>
       <c r="P142" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Revisión manual pendiente. Apoyo automatizado en EV-MVC-GEN-04-apoyo.txt y capturas EV-MVC-GEN-04-*.png: movil (375px) inicio: desborde horizontal de la página 0px; tabla con desplazamiento interno: []; movil (375px) personas-listado: desborde horizontal de la página 0px; tabla con desplazamiento interno: [True]; movil (375px) personas-crear: desborde horizontal de la página 0px; tabla con desplazamiento interno: []; movil (375px) estudios-listado: desborde horizontal de la página 0px; tabla con desplazamiento interno: [True]; movil (375px) estudios-crear: desborde horizontal de la página 0px; tabla con desplazamiento interno: []</t>
+          <t xml:space="preserve">En móvil la columna Acciones de los listados queda fuera de la vista y requiere desplazar la tabla; no hay indicación visual de que se puede desplazar. Hallazgo visual en todos los anchos: /Personas/Create:, /Profesiones/Create: muestran un recuadro de error vacío antes de enviar el formulario. Revisión asistida: confirmar el criterio con el responsable de QA. Defecto DEF-09.</t>
         </is>
       </c>
     </row>
@@ -11983,16 +12025,30 @@
       </c>
       <c r="K143" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pendiente</t>
-        </is>
-      </c>
-      <c r="L143" s="17"/>
-      <c r="M143" s="17"/>
-      <c r="N143" s="18"/>
-      <c r="O143" s="17"/>
+          <t xml:space="preserve">Aprobado</t>
+        </is>
+      </c>
+      <c r="L143" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El flujo completo (inicio, validación, alta con selectores y fecha, edición, detalle, rechazo por dependientes y eliminación) se comporta igual en: Chromium (Chrome/Edge) 156.0.8078.4: 10/10 pasos; Firefox 157.0: 10/10 pasos; WebKit (Safari) 27.2: 10/10 pasos. Sin errores de consola.</t>
+        </is>
+      </c>
+      <c r="M143" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EV-MVC-GEN-05-*.png, EV-MVC-GEN-05.txt</t>
+        </is>
+      </c>
+      <c r="N143" s="18">
+        <v>46322</v>
+      </c>
+      <c r="O143" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Automatizado</t>
+        </is>
+      </c>
       <c r="P143" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Revisión manual pendiente: repetir un flujo completo en Chrome, Edge y Firefox.</t>
+          <t xml:space="preserve">Chrome y Edge no están instalados en el equipo de pruebas; se usaron los motores de Playwright: Chromium (el de Chrome y Edge), Firefox y WebKit (el de Safari), sin interfaz grafica.</t>
         </is>
       </c>
     </row>
@@ -13313,16 +13369,30 @@
       </c>
       <c r="K166" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pendiente</t>
-        </is>
-      </c>
-      <c r="L166" s="17"/>
-      <c r="M166" s="17"/>
-      <c r="N166" s="18"/>
-      <c r="O166" s="17"/>
+          <t xml:space="preserve">Fallido</t>
+        </is>
+      </c>
+      <c r="L166" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La redacción está en tercera persona y sin voseo, pero 39 párrafos de cuerpo usan el estilo de título Heading2, hay 3 oraciones que empiezan en minúscula tras punto (sección 1.2), las secciones 3.5 y 3.7 mencionan a Codex y las referencias están marcadas como preliminares.</t>
+        </is>
+      </c>
+      <c r="M166" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EV-ENT-12.txt</t>
+        </is>
+      </c>
+      <c r="N166" s="18">
+        <v>46322</v>
+      </c>
+      <c r="O166" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Automatizado</t>
+        </is>
+      </c>
       <c r="P166" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Revisión manual pendiente sobre el documento final (estilos, ortografia, tercera persona y referencias).</t>
+          <t xml:space="preserve">Las referencias no incluyen las fuentes usadas de ASP.NET Core MVC, EF Core, SQL Server ni Swagger; la de Microsoft Learn corresponde a Entity Data Model (EF 6). Revisado sobre la copia _QA. Revisión asistida: confirmar el criterio con el responsable de QA. Defecto DEF-11.</t>
         </is>
       </c>
     </row>
@@ -14500,49 +14570,199 @@
       </c>
     </row>
     <row r="10" spans="1:13">
-      <c r="A10" s="16"/>
-      <c r="B10" s="18"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="16"/>
-      <c r="J10" s="16"/>
-      <c r="K10" s="17"/>
-      <c r="L10" s="17"/>
-      <c r="M10" s="17"/>
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEF-09</t>
+        </is>
+      </c>
+      <c r="B10" s="18">
+        <v>46322</v>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MVC-GEN-04</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R07</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Frontend MVC</t>
+        </is>
+      </c>
+      <c r="F10" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Los formularios de creación de personas y profesiones muestran un recuadro de error vacío antes de enviar.</t>
+        </is>
+      </c>
+      <c r="G10" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Abrir /Personas/Create o /Profesiones/Create sin enviar datos.</t>
+        </is>
+      </c>
+      <c r="H10" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Esperado: sin resumen de errores hasta enviar. Obtenido: div de validación con la clase validation-summary-errors y un recuadro rojo vacío de 24 px en los tres anchos.</t>
+        </is>
+      </c>
+      <c r="I10" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baja</t>
+        </is>
+      </c>
+      <c r="J10" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abierto</t>
+        </is>
+      </c>
+      <c r="K10" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Andrés</t>
+        </is>
+      </c>
+      <c r="L10" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EV-MVC-GEN-04-resumen-vacio.png, EV-MVC-GEN-04.txt</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hallazgo visual durante MVC-GEN-04; no impide usar el formulario. Causa probable: el GET de Create llama a ModelState.SetModelValue para dejar la clave vacía y el estado queda sin validar. Propuesta: quitar esa llamada (por ejemplo, mostrar la clave vacía con un DTO de vista con clave nullable) o renderizar el resumen solo si hay errores.</t>
+        </is>
+      </c>
     </row>
     <row r="11" spans="1:13">
-      <c r="A11" s="16"/>
-      <c r="B11" s="18"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
-      <c r="I11" s="16"/>
-      <c r="J11" s="16"/>
-      <c r="K11" s="17"/>
-      <c r="L11" s="17"/>
-      <c r="M11" s="17"/>
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEF-10</t>
+        </is>
+      </c>
+      <c r="B11" s="18">
+        <v>46322</v>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SW-09</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R06</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Swagger</t>
+        </is>
+      </c>
+      <c r="F11" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Swagger no muestra resumenes de las operaciones ni descripciones de parametros y campos.</t>
+        </is>
+      </c>
+      <c r="G11" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Abrir /swagger. 2. Revisar operaciones y esquemas (o swagger.json).</t>
+        </is>
+      </c>
+      <c r="H11" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Esperado: un tercero entiende y prueba la API sin explicacion adicional. Obtenido: 0 de 20 operaciones con resumen y 0 de 15 propiedades con descripción; campos como duenio, oper, nom o univer no se explican.</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baja</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abierto</t>
+        </is>
+      </c>
+      <c r="K11" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tomás</t>
+        </is>
+      </c>
+      <c r="L11" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EV-SW-09.txt, EV-SW-01.png</t>
+        </is>
+      </c>
+      <c r="M11" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Propuesta: &lt;GenerateDocumentationFile&gt;true&lt;/GenerateDocumentationFile&gt; en el .csproj, options.IncludeXmlComments(...) en AddSwaggerGen y comentarios /// en controladores y DTO (ya existen 4 en los DTO).</t>
+        </is>
+      </c>
     </row>
     <row r="12" spans="1:13">
-      <c r="A12" s="16"/>
-      <c r="B12" s="18"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="16"/>
-      <c r="J12" s="16"/>
-      <c r="K12" s="17"/>
-      <c r="L12" s="17"/>
-      <c r="M12" s="17"/>
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEF-11</t>
+        </is>
+      </c>
+      <c r="B12" s="18">
+        <v>46322</v>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ENT-12</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R11</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repositorio y entrega</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El documento mezcla estilos de título y cuerpo, tiene errores de mayusculas, menciona a Codex y sus referencias están incompletas.</t>
+        </is>
+      </c>
+      <c r="G12" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Abrir el documento y revisar estilos de parrafo, redaccion y referencias.</t>
+        </is>
+      </c>
+      <c r="H12" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Esperado: formato uniforme, tercera persona y referencias completas. Obtenido: 39 parrafos de cuerpo con estilo Heading2, oraciones en minuscula tras punto en 1.2, mencion a Codex en 3.5 y 3.7 y referencias marcadas como preliminares.</t>
+        </is>
+      </c>
+      <c r="I12" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baja</t>
+        </is>
+      </c>
+      <c r="J12" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abierto</t>
+        </is>
+      </c>
+      <c r="K12" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Andrés</t>
+        </is>
+      </c>
+      <c r="L12" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EV-ENT-12.txt</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Propuesta: aplicar Normal a los parrafos de cuerpo y un estilo de pie a las figuras, corregir las mayusculas de 1.2, decidir con el equipo si se menciona la herramienta usada y completar las referencias en APA (ASP.NET Core MVC, EF Core, SQL Server, Swashbuckle).</t>
+        </is>
+      </c>
     </row>
     <row r="13" spans="1:13">
       <c r="A13" s="16"/>

</xml_diff>

<commit_message>
docs(qa): preparar la sección 3.9 para Google Docs
Agrega el HTML de la sección 3.9 y sus figuras para insertarlos en el
documento compartido. ENT-12 pasa a revisar la versión en línea del
documento y DEF-11 se ajusta a su estado actual.
</commit_message>
<xml_diff>
--- a/QA/Matriz_Pruebas_Laboratorio1_QA.xlsx
+++ b/QA/Matriz_Pruebas_Laboratorio1_QA.xlsx
@@ -13374,7 +13374,7 @@
       </c>
       <c r="L166" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">La redacción está en tercera persona y sin voseo, pero 39 párrafos de cuerpo usan el estilo de título Heading2, hay 3 oraciones que empiezan en minúscula tras punto (sección 1.2), las secciones 3.5 y 3.7 mencionan a Codex y las referencias están marcadas como preliminares.</t>
+          <t xml:space="preserve">La redacción está en tercera persona, sin voseo y sin errores de mayúsculas, pero 38 párrafos de cuerpo usan el estilo Título 2 (aparecen como títulos en el esquema); las referencias están marcadas como preliminares.</t>
         </is>
       </c>
       <c r="M166" s="17" t="inlineStr">
@@ -13392,7 +13392,7 @@
       </c>
       <c r="P166" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Las referencias no incluyen las fuentes usadas de ASP.NET Core MVC, EF Core, SQL Server ni Swagger; la de Microsoft Learn corresponde a Entity Data Model (EF 6). Revisado sobre la copia _QA. Revisión asistida: confirmar el criterio con el responsable de QA. Defecto DEF-11.</t>
+          <t xml:space="preserve">Revisado sobre la versión en línea del documento (Google Docs). Las referencias no incluyen las fuentes de ASP.NET Core MVC, EF Core, SQL Server ni Swagger; la de Microsoft Learn corresponde a Entity Data Model (EF 6). Revisión asistida: confirmar el criterio con el responsable de QA. Defecto DEF-11.</t>
         </is>
       </c>
     </row>
@@ -14725,17 +14725,17 @@
       </c>
       <c r="F12" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">El documento mezcla estilos de título y cuerpo, tiene errores de mayusculas, menciona a Codex y sus referencias están incompletas.</t>
+          <t xml:space="preserve">El documento aplica el estilo Titulo 2 a parrafos de cuerpo y sus referencias están incompletas.</t>
         </is>
       </c>
       <c r="G12" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Abrir el documento y revisar estilos de parrafo, redaccion y referencias.</t>
+          <t xml:space="preserve">1. Abrir el documento en Google Docs y revisar el esquema, los estilos de parrafo y las referencias.</t>
         </is>
       </c>
       <c r="H12" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Esperado: formato uniforme, tercera persona y referencias completas. Obtenido: 39 parrafos de cuerpo con estilo Heading2, oraciones en minuscula tras punto en 1.2, mencion a Codex en 3.5 y 3.7 y referencias marcadas como preliminares.</t>
+          <t xml:space="preserve">Esperado: formato uniforme y referencias completas. Obtenido: 38 parrafos de cuerpo con estilo Titulo 2 (aparecen en el esquema como titulos) y referencias marcadas como preliminares.</t>
         </is>
       </c>
       <c r="I12" s="16" t="inlineStr">
@@ -14760,7 +14760,7 @@
       </c>
       <c r="M12" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Propuesta: aplicar Normal a los parrafos de cuerpo y un estilo de pie a las figuras, corregir las mayusculas de 1.2, decidir con el equipo si se menciona la herramienta usada y completar las referencias en APA (ASP.NET Core MVC, EF Core, SQL Server, Swashbuckle).</t>
+          <t xml:space="preserve">La versión en linea ya corrigio las mayusculas de 1.2 y no menciona a Codex. Propuesta: aplicar Texto normal a los parrafos de cuerpo y un estilo de pie a las figuras, y completar las referencias en APA (ASP.NET Core MVC, EF Core, SQL Server, Swashbuckle).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(qa): MVC-GEN-03 comparado con el diseño de Figma
El enlace compartido del diseño permitió comparar las 21 pantallas con
sus marcos. MVC-GEN-03 pasa de Bloqueado a Aprobado con las diferencias
registradas; DEF-07 anota que el diseño tampoco muestra la edad.
Matriz, sección 3.9 y README actualizados (150 aprobados, 2 bloqueados).
</commit_message>
<xml_diff>
--- a/QA/Matriz_Pruebas_Laboratorio1_QA.xlsx
+++ b/QA/Matriz_Pruebas_Laboratorio1_QA.xlsx
@@ -2725,7 +2725,7 @@
       </c>
       <c r="B7" s="6">
         <f>COUNTIF('Casos de prueba'!$K$2:$K$500,"Aprobado")</f>
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="B9" s="6">
         <f>COUNTIF('Casos de prueba'!$K$2:$K$500,"Bloqueado")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -2770,7 +2770,7 @@
       </c>
       <c r="B12" s="7">
         <f>IFERROR((B7+B8)/(B6-B11),0)</f>
-        <v>0.981818181818182</v>
+        <v>0.987878787878788</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -2779,7 +2779,7 @@
       </c>
       <c r="B13" s="7">
         <f>IFERROR(B7/(B7+B8),0)</f>
-        <v>0.919753086419753</v>
+        <v>0.920245398773006</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -2954,7 +2954,7 @@
       </c>
       <c r="C24" s="9">
         <f>COUNTIFS('Casos de prueba'!$C$2:$C$500,A24,'Casos de prueba'!$K$2:$K$500,"Aprobado")</f>
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D24" s="9">
         <f>COUNTIFS('Casos de prueba'!$C$2:$C$500,A24,'Casos de prueba'!$K$2:$K$500,"Fallido")</f>
@@ -2966,11 +2966,11 @@
       </c>
       <c r="F24" s="9">
         <f>COUNTIFS('Casos de prueba'!$C$2:$C$500,A24,'Casos de prueba'!$K$2:$K$500,"Bloqueado")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G24" s="10">
         <f t="shared" si="0"/>
-        <v>0.825</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -3041,7 +3041,7 @@
       </c>
       <c r="C27" s="12">
         <f>SUM(C20:C26)</f>
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D27" s="12">
         <f>SUM(D20:D26)</f>
@@ -3053,11 +3053,11 @@
       </c>
       <c r="F27" s="12">
         <f>SUM(F20:F26)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G27" s="13">
         <f t="shared" si="0"/>
-        <v>0.903030303030303</v>
+        <v>0.909090909090909</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -3425,7 +3425,7 @@
       </c>
       <c r="F8" s="15">
         <f>COUNTIFS('Casos de prueba'!$B$2:$B$500,A8,'Casos de prueba'!$K$2:$K$500,"Aprobado")</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G8" s="15">
         <f>COUNTIFS('Casos de prueba'!$B$2:$B$500,A8,'Casos de prueba'!$K$2:$K$500,"Fallido")</f>
@@ -3433,7 +3433,7 @@
       </c>
       <c r="H8" s="15">
         <f>COUNTIFS('Casos de prueba'!$B$2:$B$500,A8,'Casos de prueba'!$K$2:$K$500,"Pendiente")+COUNTIFS('Casos de prueba'!$B$2:$B$500,A8,'Casos de prueba'!$K$2:$K$500,"Bloqueado")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8" s="15" t="str">
         <f t="shared" si="0"/>
@@ -11905,17 +11905,17 @@
       </c>
       <c r="K141" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bloqueado</t>
+          <t xml:space="preserve">Aprobado</t>
         </is>
       </c>
       <c r="L141" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">No se pudo abrir el diseño de Figma desde el entorno de pruebas (requiere sesión o permiso del autor).</t>
+          <t xml:space="preserve">Las 21 pantallas siguen el diseño de Figma: menú lateral oscuro con la opción activa, título 'Módulo / Acción' con subtítulo, tarjeta blanca, campos en dos columnas, botón principal azul y confirmación de eliminación en recuadro rojo claro. Las diferencias son de texto y de controles de formulario.</t>
         </is>
       </c>
       <c r="M141" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">pantallas/EV-MVC-GEN-03-*.png, EV-MVC-GEN-03.txt</t>
+          <t xml:space="preserve">figma/EV-MVC-GEN-03-comparacion-*.png, figma/EV-MVC-GEN-03-figma-*.png, EV-MVC-GEN-03.txt</t>
         </is>
       </c>
       <c r="N141" s="18">
@@ -11928,7 +11928,7 @@
       </c>
       <c r="P141" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Las 21 capturas de las pantallas implementadas están listas. Falta el enlace compartido de Figma o las exportaciones de Andrés para completar la comparación.</t>
+          <t xml:space="preserve">Diferencias registradas en la evidencia: enlace Eliminar en los listados, títulos y preguntas de eliminación, títulos de tarjeta en singular y listas desplegables en lugar de campos de texto. El recuadro de error vacío ya está registrado como DEF-09. Revisión asistida: confirmar el criterio con el responsable de QA.</t>
         </is>
       </c>
     </row>
@@ -14500,7 +14500,7 @@
       </c>
       <c r="M8" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Propuesta: agregar &lt;th&gt;Edad&lt;/th&gt; y &lt;td&gt;@item.Edad&lt;/td&gt; en Views/Personas/Index.cshtml, o ajustar el caso si la omisión fue una decisión de diseño (comparar con Figma).</t>
+          <t xml:space="preserve">El diseño de Figma (Personas · Listado) tampoco incluye la edad, asi que la omisión sigue el diseño. Propuesta: agregar &lt;th&gt;Edad&lt;/th&gt; y &lt;td&gt;@item.Edad&lt;/td&gt; en Views/Personas/Index.cshtml, o ajustar el caso MVC-PER-01 si el equipo mantiene el diseño.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(qa): re-prueba ronda 1 de las correcciones del PR #7
Repite los casos de DEF-06, DEF-07 y DEF-09 sobre fix/def-06-07-09 (6a0edac)
y la suite completa como regresion. Agrega la seccion 3.9.7 al documento,
notas de re-prueba en la matriz (defectos en Verificado) y deja reservada
la ronda 2 de Tomas. La primera ejecucion se conserva sin cambios.
</commit_message>
<xml_diff>
--- a/QA/Matriz_Pruebas_Laboratorio1_QA.xlsx
+++ b/QA/Matriz_Pruebas_Laboratorio1_QA.xlsx
@@ -2797,7 +2797,7 @@
       </c>
       <c r="B15" s="6">
         <f>COUNTIFS(Defectos!$A$2:$A$500,"DEF-*",Defectos!$J$2:$J$500,"Abierto")+COUNTIFS(Defectos!$A$2:$A$500,"DEF-*",Defectos!$J$2:$J$500,"En corrección")</f>
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -9984,7 +9984,7 @@
       </c>
       <c r="P107" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">El listado no muestra la columna Edad; solo aparece en Detalles. El listado sin datos se revisa en MVC-GEN (base vacía). Defecto DEF-07.</t>
+          <t xml:space="preserve">El listado no muestra la columna Edad; solo aparece en Detalles. El listado sin datos se revisa en MVC-GEN (base vacía). Defecto DEF-07. Re-prueba ronda 1 (28/10/2026, Pull Request #7): Aprobado. Evidencia en reprueba/ronda-1/EV-R1-MVC-PER-01.*.</t>
         </is>
       </c>
     </row>
@@ -10212,7 +10212,7 @@
       </c>
       <c r="P111" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">NotFound() sin UseStatusCodePages; la respuesta 404 no tiene cuerpo ni navegación. Defecto DEF-06.</t>
+          <t xml:space="preserve">NotFound() sin UseStatusCodePages; la respuesta 404 no tiene cuerpo ni navegación. Defecto DEF-06. Re-prueba ronda 1 (28/10/2026, Pull Request #7): Aprobado. Evidencia en reprueba/ronda-1/EV-R1-MVC-PER-05.*.</t>
         </is>
       </c>
     </row>
@@ -10672,7 +10672,7 @@
       </c>
       <c r="P119" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">NotFound() sin UseStatusCodePages; la respuesta 404 no tiene cuerpo ni navegación. Defecto DEF-06.</t>
+          <t xml:space="preserve">NotFound() sin UseStatusCodePages; la respuesta 404 no tiene cuerpo ni navegación. Defecto DEF-06. Re-prueba ronda 1 (28/10/2026, Pull Request #7): Aprobado. Evidencia en reprueba/ronda-1/EV-R1-MVC-TEL-05.*.</t>
         </is>
       </c>
     </row>
@@ -11128,7 +11128,7 @@
       </c>
       <c r="P127" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">NotFound() sin UseStatusCodePages; la respuesta 404 no tiene cuerpo ni navegación. Defecto DEF-06.</t>
+          <t xml:space="preserve">NotFound() sin UseStatusCodePages; la respuesta 404 no tiene cuerpo ni navegación. Defecto DEF-06. Re-prueba ronda 1 (28/10/2026, Pull Request #7): Aprobado. Evidencia en reprueba/ronda-1/EV-R1-MVC-PRO-05.*.</t>
         </is>
       </c>
     </row>
@@ -11588,7 +11588,7 @@
       </c>
       <c r="P135" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">NotFound() sin UseStatusCodePages; la respuesta 404 no tiene cuerpo ni navegación. Defecto DEF-06.</t>
+          <t xml:space="preserve">NotFound() sin UseStatusCodePages; la respuesta 404 no tiene cuerpo ni navegación. Defecto DEF-06. Re-prueba ronda 1 (28/10/2026, Pull Request #7): Aprobado. Evidencia en reprueba/ronda-1/EV-R1-MVC-EST-05.*.</t>
         </is>
       </c>
     </row>
@@ -11988,7 +11988,7 @@
       </c>
       <c r="P142" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">En móvil la columna Acciones de los listados queda fuera de la vista y requiere desplazar la tabla; no hay indicación visual de que se puede desplazar. Hallazgo visual en todos los anchos: /Personas/Create:, /Profesiones/Create: muestran un recuadro de error vacío antes de enviar el formulario. Revisión asistida: confirmar el criterio con el responsable de QA. Defecto DEF-09.</t>
+          <t xml:space="preserve">En móvil la columna Acciones de los listados queda fuera de la vista y requiere desplazar la tabla; no hay indicación visual de que se puede desplazar. Hallazgo visual en todos los anchos: /Personas/Create:, /Profesiones/Create: muestran un recuadro de error vacío antes de enviar el formulario. Revisión asistida: confirmar el criterio con el responsable de QA. Defecto DEF-09. Re-prueba ronda 1 (28/10/2026, Pull Request #7): Aprobado. Evidencia en reprueba/ronda-1/EV-R1-MVC-GEN-04.*.</t>
         </is>
       </c>
     </row>
@@ -12164,7 +12164,7 @@
       </c>
       <c r="P145" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Propuesta: app.UseStatusCodePagesWithReExecute("/Home/Error") o una vista NotFound. Defecto DEF-06.</t>
+          <t xml:space="preserve">Propuesta: app.UseStatusCodePagesWithReExecute("/Home/Error") o una vista NotFound. Defecto DEF-06. Re-prueba ronda 1 (28/10/2026, Pull Request #7): Aprobado. Evidencia en reprueba/ronda-1/EV-R1-MVC-GEN-07.*.</t>
         </is>
       </c>
     </row>
@@ -13263,7 +13263,7 @@
         </is>
       </c>
       <c r="N164" s="18">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="O164" s="17" t="inlineStr">
         <is>
@@ -13323,7 +13323,7 @@
         </is>
       </c>
       <c r="N165" s="18">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="O165" s="17" t="inlineStr">
         <is>
@@ -14056,7 +14056,7 @@
         </is>
       </c>
       <c r="B2" s="18">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="C2" s="16" t="inlineStr">
         <is>
@@ -14121,7 +14121,7 @@
         </is>
       </c>
       <c r="B3" s="18">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="C3" s="16" t="inlineStr">
         <is>
@@ -14186,7 +14186,7 @@
         </is>
       </c>
       <c r="B4" s="18">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="C4" s="16" t="inlineStr">
         <is>
@@ -14251,7 +14251,7 @@
         </is>
       </c>
       <c r="B5" s="18">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
@@ -14316,7 +14316,7 @@
         </is>
       </c>
       <c r="B6" s="18">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
@@ -14381,7 +14381,7 @@
         </is>
       </c>
       <c r="B7" s="18">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
@@ -14420,7 +14420,7 @@
       </c>
       <c r="J7" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abierto</t>
+          <t xml:space="preserve">Verificado</t>
         </is>
       </c>
       <c r="K7" s="17" t="inlineStr">
@@ -14435,7 +14435,7 @@
       </c>
       <c r="M7" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Propuesta: app.UseStatusCodePagesWithReExecute("/Home/Error", "?code={0}") en Program.cs y una vista de no encontrado con el layout de la aplicación.</t>
+          <t xml:space="preserve">Propuesta: app.UseStatusCodePagesWithReExecute("/Home/Error", "?code={0}") en Program.cs y una vista de no encontrado con el layout de la aplicación. Corregido por Andrés Ortiz en el Pull Request #7 (commit 6a0edac) y verificado por QA el 28/10/2026 en la re-prueba ronda 1.</t>
         </is>
       </c>
     </row>
@@ -14446,7 +14446,7 @@
         </is>
       </c>
       <c r="B8" s="18">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>
@@ -14485,7 +14485,7 @@
       </c>
       <c r="J8" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abierto</t>
+          <t xml:space="preserve">Verificado</t>
         </is>
       </c>
       <c r="K8" s="17" t="inlineStr">
@@ -14500,7 +14500,7 @@
       </c>
       <c r="M8" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">El diseño de Figma (Personas · Listado) tampoco incluye la edad, asi que la omisión sigue el diseño. Propuesta: agregar &lt;th&gt;Edad&lt;/th&gt; y &lt;td&gt;@item.Edad&lt;/td&gt; en Views/Personas/Index.cshtml, o ajustar el caso MVC-PER-01 si el equipo mantiene el diseño.</t>
+          <t xml:space="preserve">El diseño de Figma (Personas · Listado) tampoco incluye la edad, asi que la omisión sigue el diseño. Propuesta: agregar &lt;th&gt;Edad&lt;/th&gt; y &lt;td&gt;@item.Edad&lt;/td&gt; en Views/Personas/Index.cshtml, o ajustar el caso MVC-PER-01 si el equipo mantiene el diseño. Corregido por Andrés Ortiz en el Pull Request #7 (commit 6a0edac) y verificado por QA el 28/10/2026 en la re-prueba ronda 1.</t>
         </is>
       </c>
     </row>
@@ -14511,7 +14511,7 @@
         </is>
       </c>
       <c r="B9" s="18">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
@@ -14576,7 +14576,7 @@
         </is>
       </c>
       <c r="B10" s="18">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="C10" s="16" t="inlineStr">
         <is>
@@ -14615,7 +14615,7 @@
       </c>
       <c r="J10" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abierto</t>
+          <t xml:space="preserve">Verificado</t>
         </is>
       </c>
       <c r="K10" s="17" t="inlineStr">
@@ -14630,7 +14630,7 @@
       </c>
       <c r="M10" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hallazgo visual durante MVC-GEN-04; no impide usar el formulario. Causa probable: el GET de Create llama a ModelState.SetModelValue para dejar la clave vacía y el estado queda sin validar. Propuesta: quitar esa llamada (por ejemplo, mostrar la clave vacía con un DTO de vista con clave nullable) o renderizar el resumen solo si hay errores.</t>
+          <t xml:space="preserve">Hallazgo visual durante MVC-GEN-04; no impide usar el formulario. Causa probable: el GET de Create llama a ModelState.SetModelValue para dejar la clave vacía y el estado queda sin validar. Propuesta: quitar esa llamada (por ejemplo, mostrar la clave vacía con un DTO de vista con clave nullable) o renderizar el resumen solo si hay errores. Corregido por Andrés Ortiz en el Pull Request #7 (commit 6a0edac) y verificado por QA el 28/10/2026 en la re-prueba ronda 1.</t>
         </is>
       </c>
     </row>
@@ -14641,7 +14641,7 @@
         </is>
       </c>
       <c r="B11" s="18">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
@@ -14706,7 +14706,7 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="C12" s="16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
test(qa): re-prueba ronda 2 de las correcciones de Tomas (PR #9, #10, #11)
Repite sobre main integrada (a05612c) los casos de DEF-01, DEF-02, DEF-03,
DEF-04, DEF-05 y DEF-10 y la suite completa como regresion. Completa la
ronda 2 en la seccion 3.9.7, la matriz (DEF-05 en Corregido, los demas en
Verificado) y el README de QA. Ajusta los scripts que tenian textos fijos
de la primera ejecucion o comparaban con la rama ya integrada del PR #2.
</commit_message>
<xml_diff>
--- a/QA/Matriz_Pruebas_Laboratorio1_QA.xlsx
+++ b/QA/Matriz_Pruebas_Laboratorio1_QA.xlsx
@@ -2797,7 +2797,7 @@
       </c>
       <c r="B15" s="6">
         <f>COUNTIFS(Defectos!$A$2:$A$500,"DEF-*",Defectos!$J$2:$J$500,"Abierto")+COUNTIFS(Defectos!$A$2:$A$500,"DEF-*",Defectos!$J$2:$J$500,"En corrección")</f>
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -4100,7 +4100,7 @@
       </c>
       <c r="P8" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Solo se pudo usar un entorno real (Docker). El documento (sec. 3.2) indica que en LocalDB se ejecuto el DDL quitando ALTER AUTHORIZATION ... TO sa, y el README no documenta ese ajuste. Falta repetirlo en Windows con LocalDB o Express. Defecto DEF-05.</t>
+          <t xml:space="preserve">Solo se pudo usar un entorno real (Docker). El documento (sec. 3.2) indica que en LocalDB se ejecuto el DDL quitando ALTER AUTHORIZATION ... TO sa, y el README no documenta ese ajuste. Falta repetirlo en Windows con LocalDB o Express. Defecto DEF-05. Re-prueba ronda 2 (28/10/2026, Pull Request #9, #10 y #11): Bloqueado. Evidencia en reprueba/ronda-2/EV-R2-BD-07.*.</t>
         </is>
       </c>
     </row>
@@ -4160,7 +4160,7 @@
       </c>
       <c r="P9" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Propuesta: advertir en el README y en el encabezado del DDL que re-ejecutarlo elimina los datos, o usar IF OBJECT_ID(...) IS NULL CREATE TABLE. Defecto DEF-04.</t>
+          <t xml:space="preserve">Propuesta: advertir en el README y en el encabezado del DDL que re-ejecutarlo elimina los datos, o usar IF OBJECT_ID(...) IS NULL CREATE TABLE. Defecto DEF-04. Re-prueba ronda 2 (28/10/2026, Pull Request #9, #10 y #11): Aprobado. Evidencia en reprueba/ronda-2/EV-R2-BD-08.*.</t>
         </is>
       </c>
     </row>
@@ -5668,7 +5668,7 @@
       </c>
       <c r="P35" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ejecutado como indica el README (dotnet run, entorno Development, página de excepciones del desarrollador). En Production la API devolveria la vista HTML /Home/Error. Propuesta: manejar el error en la API con ProblemDetails (503) en todos los entornos. Defecto DEF-03.</t>
+          <t xml:space="preserve">Ejecutado como indica el README (dotnet run, entorno Development, página de excepciones del desarrollador). En Production la API devolveria la vista HTML /Home/Error. Propuesta: manejar el error en la API con ProblemDetails (503) en todos los entornos. Defecto DEF-03. Re-prueba ronda 2 (28/10/2026, Pull Request #9, #10 y #11): Aprobado. Evidencia en reprueba/ronda-2/EV-R2-BK-09.*.</t>
         </is>
       </c>
     </row>
@@ -9328,7 +9328,7 @@
       </c>
       <c r="P96" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">El POST consulta ExistsAsync y luego inserta; si ambas solicitudes pasan la consulta, la segunda falla por PK y la excepción no se controla. Propuesta: capturar DbUpdateException (error 2627) y responder 409. Regresión en feature/frontend-mvc (eea9ee8): mismo resultado. Defecto DEF-01.</t>
+          <t xml:space="preserve">El POST consulta ExistsAsync y luego inserta; si ambas solicitudes pasan la consulta, la segunda falla por PK y la excepción no se controla. Propuesta: capturar DbUpdateException (error 2627) y responder 409. Regresión en feature/frontend-mvc (eea9ee8): mismo resultado. Defecto DEF-01. Re-prueba ronda 2 (28/10/2026, Pull Request #9, #10 y #11): Aprobado. Evidencia en reprueba/ronda-2/EV-R2-API-GEN-05.*.</t>
         </is>
       </c>
     </row>
@@ -9924,7 +9924,7 @@
       </c>
       <c r="P106" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">El código ya tiene 4 comentarios /// &lt;summary&gt; en los DTO, pero el proyecto no genera el archivo XML de documentación, por lo que Swagger no los muestra. Revisión asistida: confirmar el criterio con el responsable de QA. Defecto DEF-10.</t>
+          <t xml:space="preserve">El código ya tiene 4 comentarios /// &lt;summary&gt; en los DTO, pero el proyecto no genera el archivo XML de documentación, por lo que Swagger no los muestra. Revisión asistida: confirmar el criterio con el responsable de QA. Defecto DEF-10. Re-prueba ronda 2 (28/10/2026, Pull Request #9, #10 y #11): Aprobado. Evidencia en reprueba/ronda-2/EV-R2-SW-09.*.</t>
         </is>
       </c>
     </row>
@@ -12676,7 +12676,7 @@
       </c>
       <c r="P154" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">La API durante la caída responde 500 con la traza (ver BK-09).</t>
+          <t xml:space="preserve">La API durante la caída responde 500 con la traza (ver BK-09). Re-prueba ronda 2 (28/10/2026, Pull Request #9, #10 y #11): Aprobado. Evidencia en reprueba/ronda-2/EV-R2-INT-08.*.</t>
         </is>
       </c>
     </row>
@@ -13152,7 +13152,7 @@
       </c>
       <c r="P162" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Swagger queda expuesto fuera de Development porque UseSwagger/UseSwaggerUI no están condicionados al entorno en Program.cs. Defecto DEF-02.</t>
+          <t xml:space="preserve">Swagger queda expuesto fuera de Development porque UseSwagger/UseSwaggerUI no están condicionados al entorno en Program.cs. Defecto DEF-02. Re-prueba ronda 2 (28/10/2026, Pull Request #9, #10 y #11): Aprobado. Evidencia en reprueba/ronda-2/EV-R2-ENT-08.*.</t>
         </is>
       </c>
     </row>
@@ -13263,7 +13263,7 @@
         </is>
       </c>
       <c r="N164" s="18">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="O164" s="17" t="inlineStr">
         <is>
@@ -13323,7 +13323,7 @@
         </is>
       </c>
       <c r="N165" s="18">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="O165" s="17" t="inlineStr">
         <is>
@@ -14095,7 +14095,7 @@
       </c>
       <c r="J2" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abierto</t>
+          <t xml:space="preserve">Verificado</t>
         </is>
       </c>
       <c r="K2" s="17" t="inlineStr">
@@ -14110,7 +14110,7 @@
       </c>
       <c r="M2" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Causa: el controlador consulta ExistsAsync y luego inserta (condición de carrera). Propuesta: capturar DbUpdateException con SqlException.Number 2627/2601 en Create y responder 409 (mismo patron que MvcControllerBase.SaveAsync). Aplica a los 4 controladores REST.</t>
+          <t xml:space="preserve">Causa: el controlador consulta ExistsAsync y luego inserta (condición de carrera). Propuesta: capturar DbUpdateException con SqlException.Number 2627/2601 en Create y responder 409 (mismo patron que MvcControllerBase.SaveAsync). Aplica a los 4 controladores REST. Corregido por Tomás Ramírez (Pull Request #9, #10 y #11) y verificado por QA el 28/10/2026 en la re-prueba ronda 2.</t>
         </is>
       </c>
     </row>
@@ -14160,7 +14160,7 @@
       </c>
       <c r="J3" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abierto</t>
+          <t xml:space="preserve">Verificado</t>
         </is>
       </c>
       <c r="K3" s="17" t="inlineStr">
@@ -14175,7 +14175,7 @@
       </c>
       <c r="M3" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Propuesta: cambiar el README a 'cd publish &amp;&amp; ASPNETCORE_URLS=... dotnet personapi-dotnet.dll' o agregar --contentRoot publish; alternativamente indicar ConnectionStrings__PersonaDb.</t>
+          <t xml:space="preserve">Propuesta: cambiar el README a 'cd publish &amp;&amp; ASPNETCORE_URLS=... dotnet personapi-dotnet.dll' o agregar --contentRoot publish; alternativamente indicar ConnectionStrings__PersonaDb. Corregido por Tomás Ramírez (Pull Request #9, #10 y #11) y verificado por QA el 28/10/2026 en la re-prueba ronda 2.</t>
         </is>
       </c>
     </row>
@@ -14225,7 +14225,7 @@
       </c>
       <c r="J4" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abierto</t>
+          <t xml:space="preserve">Verificado</t>
         </is>
       </c>
       <c r="K4" s="17" t="inlineStr">
@@ -14240,7 +14240,7 @@
       </c>
       <c r="M4" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Se presenta en Development (página de excepciones del desarrollador). Propuesta: filtro o middleware para /api que devuelva ProblemDetails 503 ante SqlException en todos los entornos, como ya hace MvcControllerBase para las vistas.</t>
+          <t xml:space="preserve">Se presenta en Development (página de excepciones del desarrollador). Propuesta: filtro o middleware para /api que devuelva ProblemDetails 503 ante SqlException en todos los entornos, como ya hace MvcControllerBase para las vistas. Corregido por Tomás Ramírez (Pull Request #9, #10 y #11) y verificado por QA el 28/10/2026 en la re-prueba ronda 2.</t>
         </is>
       </c>
     </row>
@@ -14290,7 +14290,7 @@
       </c>
       <c r="J5" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abierto</t>
+          <t xml:space="preserve">Verificado</t>
         </is>
       </c>
       <c r="K5" s="17" t="inlineStr">
@@ -14305,7 +14305,7 @@
       </c>
       <c r="M5" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Propuesta: advertir en el README y en el encabezado de 01_ddl.sql que el script recrea las tablas, o crear las tablas solo si no existen.</t>
+          <t xml:space="preserve">Propuesta: advertir en el README y en el encabezado de 01_ddl.sql que el script recrea las tablas, o crear las tablas solo si no existen. Corregido por Tomás Ramírez (Pull Request #9, #10 y #11) y verificado por QA el 28/10/2026 en la re-prueba ronda 2.</t>
         </is>
       </c>
     </row>
@@ -14355,7 +14355,7 @@
       </c>
       <c r="J6" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abierto</t>
+          <t xml:space="preserve">Corregido</t>
         </is>
       </c>
       <c r="K6" s="17" t="inlineStr">
@@ -14370,7 +14370,7 @@
       </c>
       <c r="M6" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">No se reprodujo en LocalDB (no disponible en macOS); el fallo se reprodujo con un login sin sysadmin. Propuesta: quitar ALTER AUTHORIZATION o envolverlo en IF IS_SRVROLEMEMBER('sysadmin') = 1, y documentar LocalDB en el README.</t>
+          <t xml:space="preserve">No se reprodujo en LocalDB (no disponible en macOS); el fallo se reprodujo con un login sin sysadmin. Propuesta: quitar ALTER AUTHORIZATION o envolverlo en IF IS_SRVROLEMEMBER('sysadmin') = 1, y documentar LocalDB en el README. Corregido por Tomás Ramírez (Pull Request #9, #10 y #11) y comprobado por QA el 28/10/2026 solo en parte en la re-prueba ronda 2. Falta ejecutar BD-07 en Windows con SQL Server Express o LocalDB.</t>
         </is>
       </c>
     </row>
@@ -14435,7 +14435,7 @@
       </c>
       <c r="M7" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Propuesta: app.UseStatusCodePagesWithReExecute("/Home/Error", "?code={0}") en Program.cs y una vista de no encontrado con el layout de la aplicación. Corregido por Andrés Ortiz en el Pull Request #7 (commit 6a0edac) y verificado por QA el 28/10/2026 en la re-prueba ronda 1.</t>
+          <t xml:space="preserve">Propuesta: app.UseStatusCodePagesWithReExecute("/Home/Error", "?code={0}") en Program.cs y una vista de no encontrado con el layout de la aplicación. Corregido por Andrés Ortiz (Pull Request #7) y verificado por QA el 28/10/2026 en la re-prueba ronda 1.</t>
         </is>
       </c>
     </row>
@@ -14500,7 +14500,7 @@
       </c>
       <c r="M8" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">El diseño de Figma (Personas · Listado) tampoco incluye la edad, asi que la omisión sigue el diseño. Propuesta: agregar &lt;th&gt;Edad&lt;/th&gt; y &lt;td&gt;@item.Edad&lt;/td&gt; en Views/Personas/Index.cshtml, o ajustar el caso MVC-PER-01 si el equipo mantiene el diseño. Corregido por Andrés Ortiz en el Pull Request #7 (commit 6a0edac) y verificado por QA el 28/10/2026 en la re-prueba ronda 1.</t>
+          <t xml:space="preserve">El diseño de Figma (Personas · Listado) tampoco incluye la edad, asi que la omisión sigue el diseño. Propuesta: agregar &lt;th&gt;Edad&lt;/th&gt; y &lt;td&gt;@item.Edad&lt;/td&gt; en Views/Personas/Index.cshtml, o ajustar el caso MVC-PER-01 si el equipo mantiene el diseño. Corregido por Andrés Ortiz (Pull Request #7) y verificado por QA el 28/10/2026 en la re-prueba ronda 1.</t>
         </is>
       </c>
     </row>
@@ -14630,7 +14630,7 @@
       </c>
       <c r="M10" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hallazgo visual durante MVC-GEN-04; no impide usar el formulario. Causa probable: el GET de Create llama a ModelState.SetModelValue para dejar la clave vacía y el estado queda sin validar. Propuesta: quitar esa llamada (por ejemplo, mostrar la clave vacía con un DTO de vista con clave nullable) o renderizar el resumen solo si hay errores. Corregido por Andrés Ortiz en el Pull Request #7 (commit 6a0edac) y verificado por QA el 28/10/2026 en la re-prueba ronda 1.</t>
+          <t xml:space="preserve">Hallazgo visual durante MVC-GEN-04; no impide usar el formulario. Causa probable: el GET de Create llama a ModelState.SetModelValue para dejar la clave vacía y el estado queda sin validar. Propuesta: quitar esa llamada (por ejemplo, mostrar la clave vacía con un DTO de vista con clave nullable) o renderizar el resumen solo si hay errores. Corregido por Andrés Ortiz (Pull Request #7) y verificado por QA el 28/10/2026 en la re-prueba ronda 1.</t>
         </is>
       </c>
     </row>
@@ -14680,7 +14680,7 @@
       </c>
       <c r="J11" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abierto</t>
+          <t xml:space="preserve">Verificado</t>
         </is>
       </c>
       <c r="K11" s="17" t="inlineStr">
@@ -14695,7 +14695,7 @@
       </c>
       <c r="M11" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Propuesta: &lt;GenerateDocumentationFile&gt;true&lt;/GenerateDocumentationFile&gt; en el .csproj, options.IncludeXmlComments(...) en AddSwaggerGen y comentarios /// en controladores y DTO (ya existen 4 en los DTO).</t>
+          <t xml:space="preserve">Propuesta: &lt;GenerateDocumentationFile&gt;true&lt;/GenerateDocumentationFile&gt; en el .csproj, options.IncludeXmlComments(...) en AddSwaggerGen y comentarios /// en controladores y DTO (ya existen 4 en los DTO). Corregido por Tomás Ramírez (Pull Request #9, #10 y #11) y verificado por QA el 28/10/2026 en la re-prueba ronda 2.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(qa): DEF-12 y re-prueba ronda 3 (PR #13)
Registra DEF-12 (falta Microsoft.EntityFrameworkCore.Tools, exigido por el
enunciado) y amplia BK-01 a los tres paquetes del procedimiento: falla en
6d26734 y pasa en f68b6a5. Agrega la ronda 3 a la seccion 3.9.7, la matriz
y el README de QA. La seccion 3.9.4 conserva los 11 defectos de la primera
ejecucion y la matriz usa la fecha de deteccion de cada defecto.
</commit_message>
<xml_diff>
--- a/QA/Matriz_Pruebas_Laboratorio1_QA.xlsx
+++ b/QA/Matriz_Pruebas_Laboratorio1_QA.xlsx
@@ -2788,7 +2788,7 @@
       </c>
       <c r="B14" s="6">
         <f>COUNTIF(Defectos!$A$2:$A$500,"DEF-*")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -5188,7 +5188,7 @@
       </c>
       <c r="P27" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">.NET 6 está fuera de soporte desde noviembre de 2024; con SDK recientes se emite la advertencia NETSDK1138. Regresión en feature/frontend-mvc (eea9ee8): mismo resultado.</t>
+          <t xml:space="preserve">.NET 6 está fuera de soporte desde noviembre de 2024; con SDK recientes se emite la advertencia NETSDK1138. Regresión en feature/frontend-mvc (eea9ee8): mismo resultado. Defecto DEF-12. Re-prueba ronda 3 (29/10/2026, Pull Request #13): Aprobado. Evidencia en reprueba/ronda-3/EV-R3-BK-01.*.</t>
         </is>
       </c>
     </row>
@@ -14056,7 +14056,7 @@
         </is>
       </c>
       <c r="B2" s="18">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="C2" s="16" t="inlineStr">
         <is>
@@ -14121,7 +14121,7 @@
         </is>
       </c>
       <c r="B3" s="18">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="C3" s="16" t="inlineStr">
         <is>
@@ -14186,7 +14186,7 @@
         </is>
       </c>
       <c r="B4" s="18">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="C4" s="16" t="inlineStr">
         <is>
@@ -14251,7 +14251,7 @@
         </is>
       </c>
       <c r="B5" s="18">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
@@ -14316,7 +14316,7 @@
         </is>
       </c>
       <c r="B6" s="18">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
@@ -14381,7 +14381,7 @@
         </is>
       </c>
       <c r="B7" s="18">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
@@ -14446,7 +14446,7 @@
         </is>
       </c>
       <c r="B8" s="18">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>
@@ -14511,7 +14511,7 @@
         </is>
       </c>
       <c r="B9" s="18">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
@@ -14576,7 +14576,7 @@
         </is>
       </c>
       <c r="B10" s="18">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="C10" s="16" t="inlineStr">
         <is>
@@ -14641,7 +14641,7 @@
         </is>
       </c>
       <c r="B11" s="18">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
@@ -14706,78 +14706,128 @@
         </is>
       </c>
       <c r="B12" s="18">
+        <v>46322</v>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ENT-12</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R11</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repositorio y entrega</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El documento aplica el estilo Titulo 2 a parrafos de cuerpo y sus referencias están incompletas.</t>
+        </is>
+      </c>
+      <c r="G12" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Abrir el documento en Google Docs y revisar el esquema, los estilos de parrafo y las referencias.</t>
+        </is>
+      </c>
+      <c r="H12" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Esperado: formato uniforme y referencias completas. Obtenido: 38 parrafos de cuerpo con estilo Titulo 2 (aparecen en el esquema como titulos) y referencias marcadas como preliminares.</t>
+        </is>
+      </c>
+      <c r="I12" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baja</t>
+        </is>
+      </c>
+      <c r="J12" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abierto</t>
+        </is>
+      </c>
+      <c r="K12" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Andrés</t>
+        </is>
+      </c>
+      <c r="L12" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EV-ENT-12.txt</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La versión en linea ya corrigio las mayusculas de 1.2 y no menciona a Codex. Propuesta: aplicar Texto normal a los parrafos de cuerpo y un estilo de pie a las figuras, y completar las referencias en APA (ASP.NET Core MVC, EF Core, SQL Server, Swashbuckle).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" spans="1:13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEF-12</t>
+        </is>
+      </c>
+      <c r="B13" s="18">
         <v>46323</v>
       </c>
-      <c r="C12" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ENT-12</t>
-        </is>
-      </c>
-      <c r="D12" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R11</t>
-        </is>
-      </c>
-      <c r="E12" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Repositorio y entrega</t>
-        </is>
-      </c>
-      <c r="F12" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">El documento aplica el estilo Titulo 2 a parrafos de cuerpo y sus referencias están incompletas.</t>
-        </is>
-      </c>
-      <c r="G12" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1. Abrir el documento en Google Docs y revisar el esquema, los estilos de parrafo y las referencias.</t>
-        </is>
-      </c>
-      <c r="H12" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Esperado: formato uniforme y referencias completas. Obtenido: 38 parrafos de cuerpo con estilo Titulo 2 (aparecen en el esquema como titulos) y referencias marcadas como preliminares.</t>
-        </is>
-      </c>
-      <c r="I12" s="16" t="inlineStr">
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BK-01</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R03</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Backend y DAO</t>
+        </is>
+      </c>
+      <c r="F13" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El proyecto no incluye el paquete Microsoft.EntityFrameworkCore.Tools que exige el procedimiento del enunciado.</t>
+        </is>
+      </c>
+      <c r="G13" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Revisar los PackageReference de personapi-dotnet/personapi-dotnet.csproj. 2. Contrastar con el paso 8.8 del enunciado (Microsoft.EntityFrameworkCore, .SqlServer y .Tools).</t>
+        </is>
+      </c>
+      <c r="H13" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Esperado: los tres paquetes del enunciado. Obtenido: EntityFrameworkCore, SqlServer y Design; falta Tools, que aporta Scaffold-DbContext en la Consola del Administrador de paquetes.</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">Baja</t>
         </is>
       </c>
-      <c r="J12" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Abierto</t>
-        </is>
-      </c>
-      <c r="K12" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Andrés</t>
-        </is>
-      </c>
-      <c r="L12" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">EV-ENT-12.txt</t>
-        </is>
-      </c>
-      <c r="M12" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">La versión en linea ya corrigio las mayusculas de 1.2 y no menciona a Codex. Propuesta: aplicar Texto normal a los parrafos de cuerpo y un estilo de pie a las figuras, y completar las referencias en APA (ASP.NET Core MVC, EF Core, SQL Server, Swashbuckle).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" spans="1:13">
-      <c r="A13" s="16"/>
-      <c r="B13" s="18"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="17"/>
-      <c r="I13" s="16"/>
-      <c r="J13" s="16"/>
-      <c r="K13" s="17"/>
-      <c r="L13" s="17"/>
-      <c r="M13" s="17"/>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verificado</t>
+        </is>
+      </c>
+      <c r="K13" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tomás</t>
+        </is>
+      </c>
+      <c r="L13" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EV-BK-01.txt</t>
+        </is>
+      </c>
+      <c r="M13" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detectado al contrastar el repositorio con el enunciado oficial, recibido después de la primera ejecución; BK-01 se habia aprobado con un criterio que no incluia Tools. Propuesta: agregar Microsoft.EntityFrameworkCore.Tools 6.0.36. Corregido por Tomás Ramírez (Pull Request #13) y verificado por QA el 29/10/2026 en la re-prueba ronda 3.</t>
+        </is>
+      </c>
     </row>
     <row r="14" spans="1:13">
       <c r="A14" s="16"/>

</xml_diff>